<commit_message>
Correccion de formato de precios: regla del ultimo digito y coma
</commit_message>
<xml_diff>
--- a/precios.xlsx
+++ b/precios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josue\Documents\Proyecto_Catalogo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26BA3C25-204D-4E38-A1B7-5C8BB32F9107}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D358ACC5-D182-4BE3-90CB-83934996E988}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="6615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10766,9 +10766,7 @@
       <c r="C56" s="7">
         <v>8971045</v>
       </c>
-      <c r="D56" s="3">
-        <v>8971.0400000000009</v>
-      </c>
+      <c r="D56" s="3"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="5">
@@ -10780,9 +10778,7 @@
       <c r="C57" s="7">
         <v>8971045</v>
       </c>
-      <c r="D57" s="3">
-        <v>8971.0400000000009</v>
-      </c>
+      <c r="D57" s="3"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="5">
@@ -10794,9 +10790,7 @@
       <c r="C58" s="7">
         <v>8971045</v>
       </c>
-      <c r="D58" s="3">
-        <v>8971.0400000000009</v>
-      </c>
+      <c r="D58" s="3"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="5">
@@ -10808,9 +10802,7 @@
       <c r="C59" s="7">
         <v>8971045</v>
       </c>
-      <c r="D59" s="3">
-        <v>8971.0400000000009</v>
-      </c>
+      <c r="D59" s="3"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="5">
@@ -10822,9 +10814,7 @@
       <c r="C60" s="7">
         <v>12092390</v>
       </c>
-      <c r="D60" s="3">
-        <v>12092.39</v>
-      </c>
+      <c r="D60" s="3"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="5">
@@ -10836,9 +10826,7 @@
       <c r="C61" s="7">
         <v>8971045</v>
       </c>
-      <c r="D61" s="3">
-        <v>8971.0400000000009</v>
-      </c>
+      <c r="D61" s="3"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="5">

</xml_diff>

<commit_message>
Comprobado y forzado el formato de precios locales
</commit_message>
<xml_diff>
--- a/precios.xlsx
+++ b/precios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josue\Documents\Proyecto_Catalogo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D358ACC5-D182-4BE3-90CB-83934996E988}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5EE5FF9-006E-4A90-890E-0812FB428862}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="6615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13469,7 +13469,9 @@
       <c r="C269" s="7">
         <v>25199963</v>
       </c>
-      <c r="D269" s="3"/>
+      <c r="D269" s="3">
+        <v>1259.99</v>
+      </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A270" s="5">
@@ -13541,7 +13543,9 @@
       <c r="C275" s="7">
         <v>18999481</v>
       </c>
-      <c r="D275" s="3"/>
+      <c r="D275" s="3">
+        <v>379.98</v>
+      </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A276" s="5">
@@ -13553,7 +13557,9 @@
       <c r="C276" s="7">
         <v>18999481</v>
       </c>
-      <c r="D276" s="3"/>
+      <c r="D276" s="3">
+        <v>379.98</v>
+      </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A277" s="5">
@@ -13565,7 +13571,9 @@
       <c r="C277" s="7">
         <v>18999481</v>
       </c>
-      <c r="D277" s="3"/>
+      <c r="D277" s="3">
+        <v>379.98</v>
+      </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A278" s="5">
@@ -13577,7 +13585,9 @@
       <c r="C278" s="7">
         <v>25199963</v>
       </c>
-      <c r="D278" s="3"/>
+      <c r="D278" s="3">
+        <v>1259.99</v>
+      </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A279" s="5">
@@ -13589,7 +13599,9 @@
       <c r="C279" s="7">
         <v>25895999</v>
       </c>
-      <c r="D279" s="3"/>
+      <c r="D279" s="3">
+        <v>1259.99</v>
+      </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A280" s="5">
@@ -13601,7 +13613,9 @@
       <c r="C280" s="7">
         <v>18999481</v>
       </c>
-      <c r="D280" s="3"/>
+      <c r="D280" s="3">
+        <v>379.98</v>
+      </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A281" s="5">
@@ -13613,7 +13627,9 @@
       <c r="C281" s="7">
         <v>15750056</v>
       </c>
-      <c r="D281" s="3"/>
+      <c r="D281" s="3">
+        <v>630</v>
+      </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A282" s="5">
@@ -13977,7 +13993,9 @@
       <c r="C308" s="7">
         <v>15750056</v>
       </c>
-      <c r="D308" s="3"/>
+      <c r="D308" s="3">
+        <v>630</v>
+      </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A309" s="5">
@@ -14275,7 +14293,9 @@
       <c r="C332" s="7">
         <v>15750056</v>
       </c>
-      <c r="D332" s="3"/>
+      <c r="D332" s="3">
+        <v>630</v>
+      </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A333" s="5">
@@ -14285,9 +14305,11 @@
         <v>342</v>
       </c>
       <c r="C333" s="7">
-        <v>67499790</v>
-      </c>
-      <c r="D333" s="3"/>
+        <v>18999481</v>
+      </c>
+      <c r="D333" s="3">
+        <v>379.98</v>
+      </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A334" s="5">
@@ -14299,7 +14321,9 @@
       <c r="C334" s="7">
         <v>15750056</v>
       </c>
-      <c r="D334" s="3"/>
+      <c r="D334" s="3">
+        <v>630</v>
+      </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A335" s="5">
@@ -27504,7 +27528,7 @@
         <v>15750150</v>
       </c>
       <c r="D1414" s="3">
-        <v>567.01</v>
+        <v>630</v>
       </c>
     </row>
     <row r="1415" spans="1:4" x14ac:dyDescent="0.2">
@@ -27518,7 +27542,7 @@
         <v>18999481</v>
       </c>
       <c r="D1415" s="3">
-        <v>341.99</v>
+        <v>379.98</v>
       </c>
     </row>
     <row r="1416" spans="1:4" x14ac:dyDescent="0.2">
@@ -27791,11 +27815,9 @@
         <v>1404</v>
       </c>
       <c r="C1436" s="7">
-        <v>25199980</v>
-      </c>
-      <c r="D1436" s="3">
-        <v>1134</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D1436" s="3"/>
     </row>
     <row r="1437" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1437" s="5">
@@ -39045,7 +39067,9 @@
       <c r="C2347" s="7">
         <v>21150422</v>
       </c>
-      <c r="D2347" s="3"/>
+      <c r="D2347" s="3">
+        <v>846.01</v>
+      </c>
     </row>
     <row r="2348" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2348" s="5">
@@ -42013,7 +42037,9 @@
       <c r="C2573" s="7">
         <v>12063966</v>
       </c>
-      <c r="D2573" s="3"/>
+      <c r="D2573" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2574" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2574" s="5">
@@ -42025,7 +42051,9 @@
       <c r="C2574" s="7">
         <v>15339990</v>
       </c>
-      <c r="D2574" s="3"/>
+      <c r="D2574" s="3">
+        <v>613.59</v>
+      </c>
     </row>
     <row r="2575" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2575" s="5">
@@ -42037,7 +42065,9 @@
       <c r="C2575" s="7">
         <v>44095909</v>
       </c>
-      <c r="D2575" s="3"/>
+      <c r="D2575" s="3">
+        <v>2204.79</v>
+      </c>
     </row>
     <row r="2576" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2576" s="5">
@@ -42049,7 +42079,9 @@
       <c r="C2576" s="7">
         <v>12063966</v>
       </c>
-      <c r="D2576" s="3"/>
+      <c r="D2576" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2577" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2577" s="5">
@@ -42109,7 +42141,9 @@
       <c r="C2581" s="7">
         <v>13519998</v>
       </c>
-      <c r="D2581" s="3"/>
+      <c r="D2581" s="3">
+        <v>540.79</v>
+      </c>
     </row>
     <row r="2582" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2582" s="5">
@@ -42121,7 +42155,9 @@
       <c r="C2582" s="7">
         <v>11023993</v>
       </c>
-      <c r="D2582" s="3"/>
+      <c r="D2582" s="3">
+        <v>551.19000000000005</v>
+      </c>
     </row>
     <row r="2583" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2583" s="5">
@@ -42133,7 +42169,9 @@
       <c r="C2583" s="7">
         <v>11023993</v>
       </c>
-      <c r="D2583" s="3"/>
+      <c r="D2583" s="3">
+        <v>551.19000000000005</v>
+      </c>
     </row>
     <row r="2584" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2584" s="5">
@@ -42145,7 +42183,9 @@
       <c r="C2584" s="7">
         <v>11439989</v>
       </c>
-      <c r="D2584" s="3"/>
+      <c r="D2584" s="3">
+        <v>571.99</v>
+      </c>
     </row>
     <row r="2585" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2585" s="5">
@@ -42241,7 +42281,9 @@
       <c r="C2592" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2592" s="3"/>
+      <c r="D2592" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2593" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2593" s="5">
@@ -42253,7 +42295,9 @@
       <c r="C2593" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2593" s="3"/>
+      <c r="D2593" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2594" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2594" s="5">
@@ -42265,7 +42309,9 @@
       <c r="C2594" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2594" s="3"/>
+      <c r="D2594" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2595" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2595" s="5">
@@ -42277,7 +42323,9 @@
       <c r="C2595" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2595" s="3"/>
+      <c r="D2595" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2596" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2596" s="5">
@@ -42289,7 +42337,9 @@
       <c r="C2596" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2596" s="3"/>
+      <c r="D2596" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2597" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2597" s="5">
@@ -42301,7 +42351,9 @@
       <c r="C2597" s="7">
         <v>12063998</v>
       </c>
-      <c r="D2597" s="3"/>
+      <c r="D2597" s="3">
+        <v>603.19000000000005</v>
+      </c>
     </row>
     <row r="2598" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2598" s="5">
@@ -49150,7 +49202,9 @@
       <c r="C3155" s="7">
         <v>18507555</v>
       </c>
-      <c r="D3155" s="3"/>
+      <c r="D3155" s="3">
+        <v>700.3</v>
+      </c>
     </row>
     <row r="3156" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3156" s="5">
@@ -49162,7 +49216,9 @@
       <c r="C3156" s="7">
         <v>18507555</v>
       </c>
-      <c r="D3156" s="3"/>
+      <c r="D3156" s="3">
+        <v>700.3</v>
+      </c>
     </row>
     <row r="3157" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3157" s="5">
@@ -49174,7 +49230,9 @@
       <c r="C3157" s="7">
         <v>18507555</v>
       </c>
-      <c r="D3157" s="3"/>
+      <c r="D3157" s="3">
+        <v>700.3</v>
+      </c>
     </row>
     <row r="3158" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3158" s="5">
@@ -49186,7 +49244,9 @@
       <c r="C3158" s="7">
         <v>18507555</v>
       </c>
-      <c r="D3158" s="3"/>
+      <c r="D3158" s="3">
+        <v>700.3</v>
+      </c>
     </row>
     <row r="3159" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3159" s="5">
@@ -49258,7 +49318,9 @@
       <c r="C3164" s="7">
         <v>23538735</v>
       </c>
-      <c r="D3164" s="3"/>
+      <c r="D3164" s="3">
+        <v>941.54</v>
+      </c>
     </row>
     <row r="3165" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3165" s="5">
@@ -49294,7 +49356,9 @@
       <c r="C3167" s="7">
         <v>21398850</v>
       </c>
-      <c r="D3167" s="3"/>
+      <c r="D3167" s="3">
+        <v>855.95</v>
+      </c>
     </row>
     <row r="3168" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3168" s="5">
@@ -49330,7 +49394,9 @@
       <c r="C3170" s="7">
         <v>18507555</v>
       </c>
-      <c r="D3170" s="3"/>
+      <c r="D3170" s="3">
+        <v>700.3</v>
+      </c>
     </row>
     <row r="3171" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3171" s="5">
@@ -49560,7 +49626,9 @@
       <c r="C3189" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3189" s="3"/>
+      <c r="D3189" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3190" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3190" s="5">
@@ -49572,7 +49640,9 @@
       <c r="C3190" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3190" s="3"/>
+      <c r="D3190" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3191" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3191" s="5">
@@ -49584,7 +49654,9 @@
       <c r="C3191" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3191" s="3"/>
+      <c r="D3191" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3192" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3192" s="5">
@@ -49596,7 +49668,9 @@
       <c r="C3192" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3192" s="3"/>
+      <c r="D3192" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3193" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3193" s="5">
@@ -49608,7 +49682,9 @@
       <c r="C3193" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3193" s="3"/>
+      <c r="D3193" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3194" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3194" s="5">
@@ -49620,7 +49696,9 @@
       <c r="C3194" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3194" s="3"/>
+      <c r="D3194" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3195" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3195" s="5">
@@ -49632,7 +49710,9 @@
       <c r="C3195" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3195" s="3"/>
+      <c r="D3195" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3196" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3196" s="5">
@@ -49644,7 +49724,9 @@
       <c r="C3196" s="7">
         <v>17070075</v>
       </c>
-      <c r="D3196" s="3"/>
+      <c r="D3196" s="3">
+        <v>682.8</v>
+      </c>
     </row>
     <row r="3197" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3197" s="5">
@@ -49692,7 +49774,9 @@
       <c r="C3200" s="7">
         <v>8265510</v>
       </c>
-      <c r="D3200" s="3"/>
+      <c r="D3200" s="3">
+        <v>330.62</v>
+      </c>
     </row>
     <row r="3201" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3201" s="5">

</xml_diff>